<commit_message>
Specify ig-publisher-version in fhir-workflows.yml (#98)
Added ig-publisher-version to the FHIR workflows configuration. 53828f87962789187fa4b6b523f929cf5341914e
</commit_message>
<xml_diff>
--- a/main/ig/FRActLMCDAFHIR.xlsx
+++ b/main/ig/FRActLMCDAFHIR.xlsx
@@ -31,7 +31,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.1.0-snapsnot</t>
   </si>
   <si>
     <t>Name</t>
@@ -55,7 +55,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-13T22:26:12+00:00</t>
+    <t>2026-03-20T08:18:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>